<commit_message>
update tinh nang moi
</commit_message>
<xml_diff>
--- a/source/src/main/java/org/example/datasinhvien.xlsx
+++ b/source/src/main/java/org/example/datasinhvien.xlsx
@@ -5,27 +5,29 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KIMQUYDEV\My drive (ngokimquyai@gmail.com) (1)\data example\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\laptrinh\quanlysinhvien\source\src\main\java\org\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{443B81B5-584C-4CA0-B35F-6463C7C0A2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD24A8C9-0B6C-465C-8940-20D9467D5B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sinhvien" sheetId="4" r:id="rId1"/>
-    <sheet name="Khoa" sheetId="1" r:id="rId2"/>
-    <sheet name="Nganh" sheetId="2" r:id="rId3"/>
-    <sheet name="Lop" sheetId="3" r:id="rId4"/>
-    <sheet name="Hocphan" sheetId="7" r:id="rId5"/>
-    <sheet name="Bangdiem" sheetId="6" r:id="rId6"/>
+    <sheet name="SinhvienCNTT" sheetId="8" r:id="rId2"/>
+    <sheet name="SinhvienKetoan" sheetId="9" r:id="rId3"/>
+    <sheet name="Khoa" sheetId="1" r:id="rId4"/>
+    <sheet name="Nganh" sheetId="2" r:id="rId5"/>
+    <sheet name="Lop" sheetId="3" r:id="rId6"/>
+    <sheet name="Hocphan" sheetId="7" r:id="rId7"/>
+    <sheet name="Bangdiem" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6959" uniqueCount="2227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7181" uniqueCount="2227">
   <si>
     <t>CKCT</t>
   </si>
@@ -7063,7 +7065,7 @@
     <col min="3" max="3" width="17.5703125" customWidth="1"/>
     <col min="4" max="4" width="18.140625" customWidth="1"/>
     <col min="5" max="5" width="24.42578125" customWidth="1"/>
-    <col min="6" max="6" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -21515,6 +21517,1118 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A1D0204-AC36-4F98-8451-03087A741665}">
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>2226</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2216</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2219</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2220</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2221</v>
+      </c>
+      <c r="F1" t="s">
+        <v>2222</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2218</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="1">
+        <v>33371</v>
+      </c>
+      <c r="G2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="1">
+        <v>33837</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="1">
+        <v>34219</v>
+      </c>
+      <c r="G4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="1">
+        <v>33486</v>
+      </c>
+      <c r="G5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E6" s="1">
+        <v>33235</v>
+      </c>
+      <c r="G6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="1">
+        <v>33626</v>
+      </c>
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="1">
+        <v>33038</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" s="1">
+        <v>34965</v>
+      </c>
+      <c r="G9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="1">
+        <v>33416</v>
+      </c>
+      <c r="G10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11" t="s">
+        <v>81</v>
+      </c>
+      <c r="E11" s="1">
+        <v>33452</v>
+      </c>
+      <c r="G11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="s">
+        <v>84</v>
+      </c>
+      <c r="E12" s="1">
+        <v>33504</v>
+      </c>
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>87</v>
+      </c>
+      <c r="E13" s="1">
+        <v>33991</v>
+      </c>
+      <c r="G13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14" t="s">
+        <v>90</v>
+      </c>
+      <c r="E14" s="1">
+        <v>34274</v>
+      </c>
+      <c r="G14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E15" s="1">
+        <v>32896</v>
+      </c>
+      <c r="G15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" s="1">
+        <v>33593</v>
+      </c>
+      <c r="G16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17" t="s">
+        <v>99</v>
+      </c>
+      <c r="E17" s="1">
+        <v>32883</v>
+      </c>
+      <c r="G17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" s="1">
+        <v>33694</v>
+      </c>
+      <c r="G18" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" s="1">
+        <v>33049</v>
+      </c>
+      <c r="G19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>108</v>
+      </c>
+      <c r="E20" s="1">
+        <v>34735</v>
+      </c>
+      <c r="G20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21" t="s">
+        <v>111</v>
+      </c>
+      <c r="E21" s="1">
+        <v>34175</v>
+      </c>
+      <c r="G21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>112</v>
+      </c>
+      <c r="B22" t="s">
+        <v>113</v>
+      </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
+      <c r="D22" t="s">
+        <v>114</v>
+      </c>
+      <c r="E22" s="1">
+        <v>33510</v>
+      </c>
+      <c r="G22" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" t="s">
+        <v>116</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23" t="s">
+        <v>117</v>
+      </c>
+      <c r="E23" s="1">
+        <v>34204</v>
+      </c>
+      <c r="G23" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
+        <v>118</v>
+      </c>
+      <c r="B24" t="s">
+        <v>119</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24" t="s">
+        <v>120</v>
+      </c>
+      <c r="E24" s="1">
+        <v>34316</v>
+      </c>
+      <c r="G24" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>121</v>
+      </c>
+      <c r="B25" t="s">
+        <v>122</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25" t="s">
+        <v>123</v>
+      </c>
+      <c r="E25" s="1">
+        <v>33610</v>
+      </c>
+      <c r="G25" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" t="s">
+        <v>124</v>
+      </c>
+      <c r="B26" t="s">
+        <v>125</v>
+      </c>
+      <c r="C26">
+        <v>2</v>
+      </c>
+      <c r="D26" t="s">
+        <v>126</v>
+      </c>
+      <c r="E26" s="1">
+        <v>33059</v>
+      </c>
+      <c r="G26" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" t="s">
+        <v>127</v>
+      </c>
+      <c r="B27" t="s">
+        <v>128</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27" t="s">
+        <v>129</v>
+      </c>
+      <c r="E27" s="1">
+        <v>33521</v>
+      </c>
+      <c r="G27" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" t="s">
+        <v>130</v>
+      </c>
+      <c r="B28" t="s">
+        <v>131</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28" t="s">
+        <v>132</v>
+      </c>
+      <c r="E28" s="1">
+        <v>35017</v>
+      </c>
+      <c r="G28" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" t="s">
+        <v>134</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29" t="s">
+        <v>135</v>
+      </c>
+      <c r="E29" s="1">
+        <v>34975</v>
+      </c>
+      <c r="G29" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>136</v>
+      </c>
+      <c r="B30" t="s">
+        <v>137</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30" t="s">
+        <v>138</v>
+      </c>
+      <c r="E30" s="1">
+        <v>33109</v>
+      </c>
+      <c r="G30" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>139</v>
+      </c>
+      <c r="B31" t="s">
+        <v>140</v>
+      </c>
+      <c r="C31">
+        <v>2</v>
+      </c>
+      <c r="D31" t="s">
+        <v>141</v>
+      </c>
+      <c r="E31" s="1">
+        <v>32966</v>
+      </c>
+      <c r="G31" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3166A83-E376-44B0-9B0A-0AAC83D53953}">
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>2226</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2216</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2219</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2220</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2221</v>
+      </c>
+      <c r="F1" t="s">
+        <v>2222</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2218</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>369</v>
+      </c>
+      <c r="B2" t="s">
+        <v>370</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>371</v>
+      </c>
+      <c r="E2" s="1">
+        <v>34319</v>
+      </c>
+      <c r="G2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>372</v>
+      </c>
+      <c r="B3" t="s">
+        <v>373</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>374</v>
+      </c>
+      <c r="E3" s="1">
+        <v>34148</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>375</v>
+      </c>
+      <c r="B4" t="s">
+        <v>376</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>377</v>
+      </c>
+      <c r="E4" s="1">
+        <v>33967</v>
+      </c>
+      <c r="G4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>378</v>
+      </c>
+      <c r="B5" t="s">
+        <v>379</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>380</v>
+      </c>
+      <c r="E5" s="1">
+        <v>33284</v>
+      </c>
+      <c r="G5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>381</v>
+      </c>
+      <c r="B6" t="s">
+        <v>382</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>383</v>
+      </c>
+      <c r="E6" s="1">
+        <v>33461</v>
+      </c>
+      <c r="G6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>384</v>
+      </c>
+      <c r="B7" t="s">
+        <v>385</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>386</v>
+      </c>
+      <c r="E7" s="1">
+        <v>34318</v>
+      </c>
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>387</v>
+      </c>
+      <c r="B8" t="s">
+        <v>388</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>389</v>
+      </c>
+      <c r="E8" s="1">
+        <v>34848</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>390</v>
+      </c>
+      <c r="B9" t="s">
+        <v>391</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>392</v>
+      </c>
+      <c r="E9" s="1">
+        <v>34351</v>
+      </c>
+      <c r="G9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>393</v>
+      </c>
+      <c r="B10" t="s">
+        <v>394</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>395</v>
+      </c>
+      <c r="E10" s="1">
+        <v>33230</v>
+      </c>
+      <c r="G10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>396</v>
+      </c>
+      <c r="B11" t="s">
+        <v>397</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11" t="s">
+        <v>398</v>
+      </c>
+      <c r="E11" s="1">
+        <v>33694</v>
+      </c>
+      <c r="G11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>399</v>
+      </c>
+      <c r="B12" t="s">
+        <v>400</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>401</v>
+      </c>
+      <c r="E12" s="1">
+        <v>34961</v>
+      </c>
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>402</v>
+      </c>
+      <c r="B13" t="s">
+        <v>403</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>404</v>
+      </c>
+      <c r="E13" s="1">
+        <v>34293</v>
+      </c>
+      <c r="G13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>405</v>
+      </c>
+      <c r="B14" t="s">
+        <v>406</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>407</v>
+      </c>
+      <c r="E14" s="1">
+        <v>34877</v>
+      </c>
+      <c r="G14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>408</v>
+      </c>
+      <c r="B15" t="s">
+        <v>409</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15" t="s">
+        <v>410</v>
+      </c>
+      <c r="E15" s="1">
+        <v>34236</v>
+      </c>
+      <c r="G15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>411</v>
+      </c>
+      <c r="B16" t="s">
+        <v>412</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16" t="s">
+        <v>413</v>
+      </c>
+      <c r="E16" s="1">
+        <v>34054</v>
+      </c>
+      <c r="G16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>414</v>
+      </c>
+      <c r="B17" t="s">
+        <v>415</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17" t="s">
+        <v>416</v>
+      </c>
+      <c r="E17" s="1">
+        <v>33422</v>
+      </c>
+      <c r="G17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>417</v>
+      </c>
+      <c r="B18" t="s">
+        <v>418</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18" t="s">
+        <v>419</v>
+      </c>
+      <c r="E18" s="1">
+        <v>34940</v>
+      </c>
+      <c r="G18" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>420</v>
+      </c>
+      <c r="B19" t="s">
+        <v>421</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s">
+        <v>422</v>
+      </c>
+      <c r="E19" s="1">
+        <v>33143</v>
+      </c>
+      <c r="G19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>423</v>
+      </c>
+      <c r="B20" t="s">
+        <v>424</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20" t="s">
+        <v>425</v>
+      </c>
+      <c r="E20" s="1">
+        <v>34484</v>
+      </c>
+      <c r="G20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>426</v>
+      </c>
+      <c r="B21" t="s">
+        <v>427</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>428</v>
+      </c>
+      <c r="E21" s="1">
+        <v>33214</v>
+      </c>
+      <c r="G21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>429</v>
+      </c>
+      <c r="B22" t="s">
+        <v>430</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22" t="s">
+        <v>431</v>
+      </c>
+      <c r="E22" s="1">
+        <v>34913</v>
+      </c>
+      <c r="G22" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>432</v>
+      </c>
+      <c r="B23" t="s">
+        <v>430</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>433</v>
+      </c>
+      <c r="E23" s="1">
+        <v>34882</v>
+      </c>
+      <c r="G23" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -21656,7 +22770,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1003054F-D1C5-4CC6-B6EA-5F5536C6E101}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -21790,7 +22904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3EF989C-6B65-4A1A-AF7C-CD92DB389731}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -21822,7 +22936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00EB8B8-851F-48F8-9D02-B145917DD433}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -21919,7 +23033,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB8A8A4A-2B88-48C5-A158-92C48DE851BA}">
   <dimension ref="A1:C1991"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
cap nhat tinh nang sinhvien
</commit_message>
<xml_diff>
--- a/source/src/main/java/org/example/datasinhvien.xlsx
+++ b/source/src/main/java/org/example/datasinhvien.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\laptrinh\quanlysinhvien\source\src\main\java\org\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD24A8C9-0B6C-465C-8940-20D9467D5B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A986DF0-2B9C-4D83-9050-14F533D60599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sinhvien" sheetId="4" r:id="rId1"/>
@@ -22,12 +22,12 @@
     <sheet name="Hocphan" sheetId="7" r:id="rId7"/>
     <sheet name="Bangdiem" sheetId="6" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7181" uniqueCount="2227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7185" uniqueCount="2229">
   <si>
     <t>CKCT</t>
   </si>
@@ -6708,6 +6708,12 @@
   </si>
   <si>
     <t>id</t>
+  </si>
+  <si>
+    <t>diemjava</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diemweb </t>
   </si>
 </sst>
 </file>
@@ -21518,13 +21524,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A1D0204-AC36-4F98-8451-03087A741665}">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="2" max="2" width="29.7109375" customWidth="1"/>
     <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>2226</v>
       </c>
@@ -21546,8 +21554,14 @@
       <c r="G1" t="s">
         <v>2218</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" t="s">
+        <v>2227</v>
+      </c>
+      <c r="I1" t="s">
+        <v>2228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -21566,8 +21580,14 @@
       <c r="G2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>55</v>
       </c>
@@ -21586,8 +21606,14 @@
       <c r="G3" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -21606,8 +21632,14 @@
       <c r="G4" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4">
+        <v>9</v>
+      </c>
+      <c r="I4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>61</v>
       </c>
@@ -21626,8 +21658,14 @@
       <c r="G5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>64</v>
       </c>
@@ -21646,8 +21684,14 @@
       <c r="G6" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>67</v>
       </c>
@@ -21666,8 +21710,14 @@
       <c r="G7" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="H7">
+        <v>9</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>70</v>
       </c>
@@ -21686,8 +21736,14 @@
       <c r="G8" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="H8">
+        <v>6</v>
+      </c>
+      <c r="I8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>73</v>
       </c>
@@ -21706,8 +21762,14 @@
       <c r="G9" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="H9">
+        <v>10</v>
+      </c>
+      <c r="I9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>76</v>
       </c>
@@ -21726,8 +21788,14 @@
       <c r="G10" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="H10">
+        <v>7</v>
+      </c>
+      <c r="I10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -21746,8 +21814,14 @@
       <c r="G11" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="H11">
+        <v>8</v>
+      </c>
+      <c r="I11">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
         <v>82</v>
       </c>
@@ -21766,8 +21840,14 @@
       <c r="G12" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="H12">
+        <v>4</v>
+      </c>
+      <c r="I12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>85</v>
       </c>
@@ -21786,8 +21866,14 @@
       <c r="G13" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="H13">
+        <v>9</v>
+      </c>
+      <c r="I13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
         <v>88</v>
       </c>
@@ -21806,8 +21892,14 @@
       <c r="G14" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="H14">
+        <v>9</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
         <v>91</v>
       </c>
@@ -21826,8 +21918,14 @@
       <c r="G15" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
         <v>94</v>
       </c>
@@ -21846,8 +21944,14 @@
       <c r="G16" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="H16">
+        <v>9</v>
+      </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>97</v>
       </c>
@@ -21866,8 +21970,14 @@
       <c r="G17" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>100</v>
       </c>
@@ -21886,8 +21996,14 @@
       <c r="G18" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="H18">
+        <v>5</v>
+      </c>
+      <c r="I18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>103</v>
       </c>
@@ -21906,8 +22022,14 @@
       <c r="G19" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="H19">
+        <v>3</v>
+      </c>
+      <c r="I19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>106</v>
       </c>
@@ -21926,8 +22048,14 @@
       <c r="G20" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="H20">
+        <v>7</v>
+      </c>
+      <c r="I20">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>109</v>
       </c>
@@ -21946,8 +22074,14 @@
       <c r="G21" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="H21">
+        <v>8</v>
+      </c>
+      <c r="I21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>112</v>
       </c>
@@ -21966,8 +22100,14 @@
       <c r="G22" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="H22">
+        <v>9</v>
+      </c>
+      <c r="I22">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
         <v>115</v>
       </c>
@@ -21986,8 +22126,14 @@
       <c r="G23" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="H23">
+        <v>7</v>
+      </c>
+      <c r="I23">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>118</v>
       </c>
@@ -22006,8 +22152,14 @@
       <c r="G24" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="H24">
+        <v>7</v>
+      </c>
+      <c r="I24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
         <v>121</v>
       </c>
@@ -22026,8 +22178,14 @@
       <c r="G25" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="26" spans="1:7">
+      <c r="H25">
+        <v>8</v>
+      </c>
+      <c r="I25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>124</v>
       </c>
@@ -22046,8 +22204,14 @@
       <c r="G26" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="27" spans="1:7">
+      <c r="H26">
+        <v>10</v>
+      </c>
+      <c r="I26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>127</v>
       </c>
@@ -22066,8 +22230,14 @@
       <c r="G27" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="H27">
+        <v>9</v>
+      </c>
+      <c r="I27">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>130</v>
       </c>
@@ -22086,8 +22256,14 @@
       <c r="G28" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="29" spans="1:7">
+      <c r="H28">
+        <v>2</v>
+      </c>
+      <c r="I28">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>133</v>
       </c>
@@ -22106,8 +22282,14 @@
       <c r="G29" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="H29">
+        <v>1</v>
+      </c>
+      <c r="I29">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>136</v>
       </c>
@@ -22126,8 +22308,14 @@
       <c r="G30" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="H30">
+        <v>4</v>
+      </c>
+      <c r="I30">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>139</v>
       </c>
@@ -22145,6 +22333,12 @@
       </c>
       <c r="G31" t="s">
         <v>50</v>
+      </c>
+      <c r="H31">
+        <v>6</v>
+      </c>
+      <c r="I31">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -22154,13 +22348,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3166A83-E376-44B0-9B0A-0AAC83D53953}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>2226</v>
       </c>
@@ -22182,8 +22376,14 @@
       <c r="G1" t="s">
         <v>2218</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" t="s">
+        <v>2227</v>
+      </c>
+      <c r="I1" t="s">
+        <v>2228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>369</v>
       </c>
@@ -22202,8 +22402,14 @@
       <c r="G2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2">
+        <v>8</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>372</v>
       </c>
@@ -22222,8 +22428,14 @@
       <c r="G3" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>375</v>
       </c>
@@ -22242,8 +22454,14 @@
       <c r="G4" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4">
+        <v>9</v>
+      </c>
+      <c r="I4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>378</v>
       </c>
@@ -22262,8 +22480,14 @@
       <c r="G5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>381</v>
       </c>
@@ -22282,8 +22506,14 @@
       <c r="G6" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>384</v>
       </c>
@@ -22302,8 +22532,14 @@
       <c r="G7" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="H7">
+        <v>9</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>387</v>
       </c>
@@ -22322,8 +22558,14 @@
       <c r="G8" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="H8">
+        <v>6</v>
+      </c>
+      <c r="I8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>390</v>
       </c>
@@ -22342,8 +22584,14 @@
       <c r="G9" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="H9">
+        <v>10</v>
+      </c>
+      <c r="I9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>393</v>
       </c>
@@ -22362,8 +22610,14 @@
       <c r="G10" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="H10">
+        <v>7</v>
+      </c>
+      <c r="I10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>396</v>
       </c>
@@ -22382,8 +22636,14 @@
       <c r="G11" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="H11">
+        <v>8</v>
+      </c>
+      <c r="I11">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
         <v>399</v>
       </c>
@@ -22402,8 +22662,14 @@
       <c r="G12" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="H12">
+        <v>4</v>
+      </c>
+      <c r="I12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>402</v>
       </c>
@@ -22422,8 +22688,14 @@
       <c r="G13" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="H13">
+        <v>9</v>
+      </c>
+      <c r="I13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
         <v>405</v>
       </c>
@@ -22442,8 +22714,14 @@
       <c r="G14" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="H14">
+        <v>9</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
         <v>408</v>
       </c>
@@ -22462,8 +22740,14 @@
       <c r="G15" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
         <v>411</v>
       </c>
@@ -22482,8 +22766,14 @@
       <c r="G16" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="H16">
+        <v>9</v>
+      </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>414</v>
       </c>
@@ -22502,8 +22792,14 @@
       <c r="G17" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>417</v>
       </c>
@@ -22522,8 +22818,14 @@
       <c r="G18" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="H18">
+        <v>5</v>
+      </c>
+      <c r="I18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>420</v>
       </c>
@@ -22542,8 +22844,14 @@
       <c r="G19" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="H19">
+        <v>3</v>
+      </c>
+      <c r="I19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>423</v>
       </c>
@@ -22562,8 +22870,14 @@
       <c r="G20" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="H20">
+        <v>7</v>
+      </c>
+      <c r="I20">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>426</v>
       </c>
@@ -22582,8 +22896,14 @@
       <c r="G21" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="H21">
+        <v>8</v>
+      </c>
+      <c r="I21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>429</v>
       </c>
@@ -22602,8 +22922,14 @@
       <c r="G22" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="H22">
+        <v>9</v>
+      </c>
+      <c r="I22">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
         <v>432</v>
       </c>
@@ -22621,6 +22947,12 @@
       </c>
       <c r="G23" t="s">
         <v>50</v>
+      </c>
+      <c r="H23">
+        <v>7</v>
+      </c>
+      <c r="I23">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>